<commit_message>
Update MLB hitter fantasy scores 2026-09-07 (2026-09-07 01:24 AM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V6_TOP30_2026_09_07.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V6_TOP30_2026_09_07.xlsx
@@ -4791,10 +4791,10 @@
         <v>9.75</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>7.24</v>
@@ -4806,13 +4806,13 @@
         <v>7.71</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>8.460000000000001</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="Q5" s="3" t="n">
         <v>7.71</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>0.911</v>
+        <v>0.91</v>
       </c>
       <c r="S5" s="3" t="n">
         <v>10.8</v>
@@ -4842,16 +4842,16 @@
         <v>78.09999999999999</v>
       </c>
       <c r="Z5" s="5" t="n">
-        <v>69.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AA5" s="5" t="n">
-        <v>69.8</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>66.09999999999999</v>
+        <v>66.3</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>66.09999999999999</v>
+        <v>66.3</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>59.9</v>
@@ -4863,10 +4863,10 @@
         <v>53.7</v>
       </c>
       <c r="AG5" s="7" t="n">
-        <v>51.9</v>
+        <v>51.8</v>
       </c>
       <c r="AH5" s="7" t="n">
-        <v>49</v>
+        <v>48.9</v>
       </c>
       <c r="AI5" s="7" t="n">
         <v>45.6</v>
@@ -4878,16 +4878,16 @@
         <v>41.6</v>
       </c>
       <c r="AL5" s="8" t="n">
-        <v>39.4</v>
+        <v>39.3</v>
       </c>
       <c r="AM5" s="8" t="n">
         <v>37.4</v>
       </c>
       <c r="AN5" s="8" t="n">
-        <v>33.2</v>
+        <v>33.1</v>
       </c>
       <c r="AO5" s="8" t="n">
-        <v>33.2</v>
+        <v>33.1</v>
       </c>
       <c r="AP5" s="8" t="n">
         <v>31.4</v>
@@ -4914,13 +4914,13 @@
         <v>21.8</v>
       </c>
       <c r="AX5" s="8" t="n">
-        <v>21.1</v>
+        <v>21</v>
       </c>
       <c r="AY5" s="8" t="n">
         <v>20.1</v>
       </c>
       <c r="AZ5" s="3" t="n">
-        <v>245</v>
+        <v>245.13</v>
       </c>
       <c r="BA5" s="4" t="inlineStr">
         <is>
@@ -4944,7 +4944,7 @@
         <v>59.9</v>
       </c>
       <c r="BF5" s="3" t="n">
-        <v>4.7</v>
+        <v>4.71</v>
       </c>
       <c r="BG5" s="3" t="n">
         <v>19.8</v>
@@ -5043,13 +5043,13 @@
         <v>1.065</v>
       </c>
       <c r="CI5" s="3" t="n">
-        <v>95.09999999999999</v>
+        <v>94.2</v>
       </c>
       <c r="CJ5" s="3" t="n">
-        <v>12.2</v>
+        <v>11.9</v>
       </c>
       <c r="CK5" s="3" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="CL5" s="3" t="n">
         <v>2</v>
@@ -5307,19 +5307,19 @@
         <v>16.5</v>
       </c>
       <c r="FM5" s="3" t="n">
-        <v>0.992</v>
+        <v>0.9918</v>
       </c>
       <c r="FN5" s="3" t="n">
         <v>0.9968</v>
       </c>
       <c r="FO5" s="3" t="n">
-        <v>1.0168</v>
+        <v>1.0167</v>
       </c>
       <c r="FP5" s="3" t="n">
         <v>1.0542</v>
       </c>
       <c r="FQ5" s="3" t="n">
-        <v>0.9438</v>
+        <v>0.9437</v>
       </c>
       <c r="FR5" s="3" t="n">
         <v>0.9811</v>
@@ -5379,7 +5379,7 @@
         <v>27</v>
       </c>
       <c r="GI5" s="3" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.9903</v>
       </c>
       <c r="GJ5" s="3" t="n">
         <v>0.1575</v>
@@ -5432,13 +5432,13 @@
         <v>7.71</v>
       </c>
       <c r="GZ5" s="3" t="n">
-        <v>3.6</v>
+        <v>3.61</v>
       </c>
       <c r="HA5" s="3" t="n">
-        <v>13.62</v>
+        <v>13.61</v>
       </c>
       <c r="HB5" s="3" t="n">
-        <v>19.99</v>
+        <v>19.98</v>
       </c>
       <c r="HC5" s="3" t="n">
         <v>4.58</v>
@@ -5455,19 +5455,19 @@
         <v>87</v>
       </c>
       <c r="HG5" s="3" t="n">
-        <v>80.7</v>
+        <v>80.8</v>
       </c>
       <c r="HH5" s="3" t="n">
-        <v>80.7</v>
+        <v>80.8</v>
       </c>
       <c r="HI5" s="3" t="n">
-        <v>72.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="HJ5" s="3" t="n">
-        <v>72.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="HK5" s="3" t="n">
-        <v>68.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="HL5" s="3" t="n">
         <v>58.8</v>
@@ -5476,31 +5476,31 @@
         <v>58.8</v>
       </c>
       <c r="HN5" s="3" t="n">
-        <v>55.5</v>
+        <v>55.4</v>
       </c>
       <c r="HO5" s="3" t="n">
-        <v>55.5</v>
+        <v>55.4</v>
       </c>
       <c r="HP5" s="3" t="n">
-        <v>48.6</v>
+        <v>48.5</v>
       </c>
       <c r="HQ5" s="3" t="n">
-        <v>48.6</v>
+        <v>48.5</v>
       </c>
       <c r="HR5" s="3" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="HS5" s="3" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="HT5" s="3" t="n">
-        <v>40.6</v>
+        <v>40.5</v>
       </c>
       <c r="HU5" s="3" t="n">
-        <v>36.7</v>
+        <v>36.6</v>
       </c>
       <c r="HV5" s="3" t="n">
-        <v>36.7</v>
+        <v>36.6</v>
       </c>
       <c r="HW5" s="3" t="n">
         <v>34.3</v>
@@ -5527,7 +5527,7 @@
         <v>24.8</v>
       </c>
       <c r="IE5" s="3" t="n">
-        <v>23.7</v>
+        <v>23.6</v>
       </c>
       <c r="IF5" s="3" t="n">
         <v>20.5</v>
@@ -10070,10 +10070,10 @@
         <v>76.5</v>
       </c>
       <c r="Z11" s="5" t="n">
-        <v>66.3</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="AA11" s="5" t="n">
-        <v>66.3</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="AB11" s="5" t="n">
         <v>60.5</v>
@@ -10085,16 +10085,16 @@
         <v>52.7</v>
       </c>
       <c r="AE11" s="7" t="n">
-        <v>48.2</v>
+        <v>48.1</v>
       </c>
       <c r="AF11" s="7" t="n">
         <v>46.7</v>
       </c>
       <c r="AG11" s="7" t="n">
-        <v>44.6</v>
+        <v>44.5</v>
       </c>
       <c r="AH11" s="7" t="n">
-        <v>41.6</v>
+        <v>41.5</v>
       </c>
       <c r="AI11" s="8" t="n">
         <v>37.7</v>
@@ -10118,7 +10118,7 @@
         <v>26.6</v>
       </c>
       <c r="AP11" s="8" t="n">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="AQ11" s="8" t="n">
         <v>23.2</v>
@@ -10148,7 +10148,7 @@
         <v>14</v>
       </c>
       <c r="AZ11" s="3" t="n">
-        <v>206.13</v>
+        <v>206.12</v>
       </c>
       <c r="BA11" s="4" t="inlineStr">
         <is>
@@ -10271,13 +10271,13 @@
         <v>1.065</v>
       </c>
       <c r="CI11" s="3" t="n">
-        <v>95.09999999999999</v>
+        <v>94.2</v>
       </c>
       <c r="CJ11" s="3" t="n">
-        <v>12.2</v>
+        <v>11.9</v>
       </c>
       <c r="CK11" s="3" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="CL11" s="3" t="n">
         <v>2</v>
@@ -10415,7 +10415,7 @@
         <v>7.72</v>
       </c>
       <c r="EA11" s="3" t="n">
-        <v>7.83</v>
+        <v>7.82</v>
       </c>
       <c r="EB11" s="3" t="n">
         <v>7.8</v>
@@ -10535,19 +10535,19 @@
         <v>16.7</v>
       </c>
       <c r="FM11" s="3" t="n">
-        <v>0.9895</v>
+        <v>0.9893</v>
       </c>
       <c r="FN11" s="3" t="n">
         <v>0.9964</v>
       </c>
       <c r="FO11" s="3" t="n">
-        <v>1.0128</v>
+        <v>1.0126</v>
       </c>
       <c r="FP11" s="3" t="n">
         <v>1.0534</v>
       </c>
       <c r="FQ11" s="3" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.9389</v>
       </c>
       <c r="FR11" s="3" t="n">
         <v>1.0058</v>
@@ -10607,7 +10607,7 @@
         <v>27</v>
       </c>
       <c r="GI11" s="3" t="n">
-        <v>0.9983</v>
+        <v>0.9982</v>
       </c>
       <c r="GJ11" s="3" t="n">
         <v>0.1498</v>
@@ -10683,10 +10683,10 @@
         <v>85.09999999999999</v>
       </c>
       <c r="HG11" s="3" t="n">
-        <v>75.40000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="HH11" s="3" t="n">
-        <v>75.40000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="HI11" s="3" t="n">
         <v>66.09999999999999</v>
@@ -10698,16 +10698,16 @@
         <v>60.7</v>
       </c>
       <c r="HL11" s="3" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="HM11" s="3" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="HN11" s="3" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="HO11" s="3" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="HP11" s="3" t="n">
         <v>39.2</v>
@@ -10731,7 +10731,7 @@
         <v>27.2</v>
       </c>
       <c r="HW11" s="3" t="n">
-        <v>25</v>
+        <v>24.9</v>
       </c>
       <c r="HX11" s="3" t="n">
         <v>22.4</v>
@@ -11154,7 +11154,7 @@
         <v>158</v>
       </c>
       <c r="CL12" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CM12" s="4" t="inlineStr">
         <is>
@@ -12028,7 +12028,7 @@
         <v>158</v>
       </c>
       <c r="CL13" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CM13" s="4" t="inlineStr">
         <is>
@@ -16901,22 +16901,22 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Jackson Merrill</t>
+          <t>Jac Caglianone</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>KC</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>WSH @ SD</t>
+          <t>ARI @ KC</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -16926,178 +16926,178 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="J19" s="3" t="n">
-        <v>7.79</v>
+        <v>8.42</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>6.87</v>
+        <v>6.92</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>6.87</v>
+        <v>6.92</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>5.15</v>
+        <v>4.37</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>7.58</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>7.03</v>
+        <v>8.68</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>7.65</v>
+        <v>7.66</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>7.03</v>
+        <v>8.35</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>0.919</v>
+        <v>1.133</v>
       </c>
       <c r="S19" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="T19" s="3" t="n">
-        <v>7.1</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>7.07</v>
+        <v>8.67</v>
       </c>
       <c r="V19" s="4" t="inlineStr">
         <is>
-          <t>0|2|0|0|8</t>
+          <t>5|0|14|9|2</t>
         </is>
       </c>
       <c r="W19" s="4" t="inlineStr">
         <is>
-          <t>0|2|0|0|8|12|5|2|23|19</t>
+          <t>5|0|14|9|2|7|8|6|42|0</t>
         </is>
       </c>
       <c r="X19" s="4" t="inlineStr">
         <is>
-          <t>0|2|0|0|8|12|5|2|23|19|0|0|14|21|0</t>
-        </is>
-      </c>
-      <c r="Y19" s="5" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="Z19" s="5" t="n">
-        <v>59.1</v>
-      </c>
-      <c r="AA19" s="6" t="n">
-        <v>54.6</v>
+          <t>5|0|14|9|2|7|8|6|42|0|7|0|5|10|15</t>
+        </is>
+      </c>
+      <c r="Y19" s="6" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="Z19" s="7" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="AA19" s="7" t="n">
+        <v>52.3</v>
       </c>
       <c r="AB19" s="7" t="n">
-        <v>53.7</v>
+        <v>50.5</v>
       </c>
       <c r="AC19" s="7" t="n">
-        <v>52</v>
+        <v>45.5</v>
       </c>
       <c r="AD19" s="7" t="n">
-        <v>48.1</v>
+        <v>43.8</v>
       </c>
       <c r="AE19" s="7" t="n">
-        <v>42.9</v>
+        <v>43.8</v>
       </c>
       <c r="AF19" s="7" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="AG19" s="8" t="n">
-        <v>39.8</v>
+        <v>40.8</v>
+      </c>
+      <c r="AG19" s="7" t="n">
+        <v>40.6</v>
       </c>
       <c r="AH19" s="8" t="n">
-        <v>34</v>
+        <v>34.6</v>
       </c>
       <c r="AI19" s="8" t="n">
-        <v>34</v>
+        <v>34.6</v>
       </c>
       <c r="AJ19" s="8" t="n">
-        <v>30.7</v>
+        <v>31.2</v>
       </c>
       <c r="AK19" s="8" t="n">
-        <v>30.7</v>
+        <v>31.2</v>
       </c>
       <c r="AL19" s="8" t="n">
-        <v>28.2</v>
+        <v>28.6</v>
       </c>
       <c r="AM19" s="8" t="n">
-        <v>28.1</v>
+        <v>28.5</v>
       </c>
       <c r="AN19" s="8" t="n">
-        <v>24.8</v>
+        <v>27.2</v>
       </c>
       <c r="AO19" s="8" t="n">
         <v>24.8</v>
       </c>
       <c r="AP19" s="8" t="n">
-        <v>22.8</v>
+        <v>23.5</v>
       </c>
       <c r="AQ19" s="8" t="n">
-        <v>22.8</v>
+        <v>23.3</v>
       </c>
       <c r="AR19" s="8" t="n">
-        <v>20.8</v>
+        <v>22.5</v>
       </c>
       <c r="AS19" s="8" t="n">
-        <v>20.8</v>
+        <v>20.9</v>
       </c>
       <c r="AT19" s="8" t="n">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="AU19" s="8" t="n">
-        <v>18.3</v>
+        <v>19.6</v>
       </c>
       <c r="AV19" s="8" t="n">
-        <v>16.2</v>
+        <v>17.9</v>
       </c>
       <c r="AW19" s="8" t="n">
-        <v>16.2</v>
+        <v>17.9</v>
       </c>
       <c r="AX19" s="8" t="n">
-        <v>16.2</v>
+        <v>16.3</v>
       </c>
       <c r="AY19" s="8" t="n">
-        <v>13.6</v>
+        <v>16.3</v>
       </c>
       <c r="AZ19" s="3" t="n">
-        <v>188.76</v>
+        <v>188.47</v>
       </c>
       <c r="BA19" s="4" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="BB19" s="9" t="inlineStr">
-        <is>
-          <t>MORE 3.0 | 59.1% | Edge +3.9</t>
+      <c r="BB19" s="10" t="inlineStr">
+        <is>
+          <t>LESS 7.5 | 65.4% | Edge +0.6</t>
         </is>
       </c>
       <c r="BC19" s="4" t="inlineStr">
         <is>
-          <t>MORE</t>
+          <t>LESS</t>
         </is>
       </c>
       <c r="BD19" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="BE19" s="3" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="BF19" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="BG19" s="3" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="BH19" s="4" t="inlineStr">
+        <is>
+          <t>Playable</t>
+        </is>
+      </c>
+      <c r="BI19" s="3" t="n">
         <v>3</v>
-      </c>
-      <c r="BE19" s="3" t="n">
-        <v>59.1</v>
-      </c>
-      <c r="BF19" s="3" t="n">
-        <v>3.87</v>
-      </c>
-      <c r="BG19" s="3" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="BH19" s="4" t="inlineStr">
-        <is>
-          <t>Playable</t>
-        </is>
-      </c>
-      <c r="BI19" s="3" t="n">
-        <v>5</v>
       </c>
       <c r="BJ19" s="4" t="inlineStr">
         <is>
@@ -17106,24 +17106,24 @@
       </c>
       <c r="BK19" s="4" t="n"/>
       <c r="BL19" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="BM19" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="BN19" s="4" t="inlineStr">
         <is>
-          <t>5-5-5-3-5-5-5</t>
+          <t>3-3-3-3-3-3</t>
         </is>
       </c>
       <c r="BO19" s="3" t="n">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="BP19" s="3" t="n">
         <v>97</v>
       </c>
       <c r="BQ19" s="3" t="n">
-        <v>4.13</v>
+        <v>4.12</v>
       </c>
       <c r="BR19" s="4" t="inlineStr">
         <is>
@@ -17131,14 +17131,14 @@
         </is>
       </c>
       <c r="BS19" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="BT19" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="BU19" s="4" t="inlineStr">
         <is>
-          <t>Jake Irvin</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="BV19" s="4" t="inlineStr">
@@ -17147,124 +17147,124 @@
         </is>
       </c>
       <c r="BW19" s="3" t="n">
-        <v>5.57</v>
+        <v>4.2</v>
       </c>
       <c r="BX19" s="3" t="n">
-        <v>1.4</v>
+        <v>1.25</v>
       </c>
       <c r="BY19" s="3" t="n">
-        <v>0.2105</v>
+        <v>0.224</v>
       </c>
       <c r="BZ19" s="3" t="n">
-        <v>0.0395</v>
+        <v>0.03</v>
       </c>
       <c r="CA19" s="3" t="n">
-        <v>0.1053</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="CB19" s="3" t="n">
-        <v>4.72</v>
+        <v>4.13</v>
       </c>
       <c r="CC19" s="3" t="n">
-        <v>1.39</v>
+        <v>1.28</v>
       </c>
       <c r="CD19" s="3" t="n">
-        <v>0.2243</v>
+        <v>0.2235</v>
       </c>
       <c r="CE19" s="3" t="n">
-        <v>0.0351</v>
+        <v>0.03</v>
       </c>
       <c r="CF19" s="4" t="inlineStr">
         <is>
-          <t>Petco Park</t>
+          <t>Kauffman Stadium</t>
         </is>
       </c>
       <c r="CG19" s="3" t="n">
-        <v>0.88</v>
+        <v>1.072</v>
       </c>
       <c r="CH19" s="3" t="n">
-        <v>1.065</v>
+        <v>1.03</v>
       </c>
       <c r="CI19" s="3" t="n">
-        <v>95.09999999999999</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="CJ19" s="3" t="n">
-        <v>12.2</v>
+        <v>8.4</v>
       </c>
       <c r="CK19" s="3" t="n">
-        <v>320</v>
+        <v>158</v>
       </c>
       <c r="CL19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM19" s="4" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="CN19" s="3" t="n">
+        <v>510</v>
+      </c>
+      <c r="CO19" s="3" t="n">
+        <v>474</v>
+      </c>
+      <c r="CP19" s="3" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="CQ19" s="3" t="n">
+        <v>0.331</v>
+      </c>
+      <c r="CR19" s="3" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="CS19" s="3" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="CT19" s="3" t="n">
+        <v>355</v>
+      </c>
+      <c r="CU19" s="3" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="CV19" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="CW19" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="CX19" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="CM19" s="4" t="inlineStr">
-        <is>
-          <t>hot, light wind</t>
-        </is>
-      </c>
-      <c r="CN19" s="3" t="n">
-        <v>587</v>
-      </c>
-      <c r="CO19" s="3" t="n">
-        <v>540</v>
-      </c>
-      <c r="CP19" s="3" t="n">
-        <v>0.237</v>
-      </c>
-      <c r="CQ19" s="3" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="CR19" s="3" t="n">
-        <v>0.411</v>
-      </c>
-      <c r="CS19" s="3" t="n">
-        <v>0.701</v>
-      </c>
-      <c r="CT19" s="3" t="n">
-        <v>421</v>
-      </c>
-      <c r="CU19" s="3" t="n">
-        <v>0.699</v>
-      </c>
-      <c r="CV19" s="3" t="n">
-        <v>128</v>
-      </c>
-      <c r="CW19" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="CX19" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="CY19" s="3" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="CZ19" s="3" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="DA19" s="3" t="n">
         <v>70</v>
       </c>
       <c r="DB19" s="3" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="DC19" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="DD19" s="3" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="DE19" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06 vs New York Yankees: 0 FS|2026-09-05 vs New York Yankees: 2 FS|2026-09-04 vs New York Yankees: 0 FS|2026-09-02 @ Cincinnati Reds: 0 FS|2026-09-01 @ Cincinnati Reds: 8 FS</t>
+          <t>2026-09-05 vs Toronto Blue Jays: 5 FS|2026-09-04 vs Toronto Blue Jays: 0 FS|2026-09-03 vs Miami Marlins: 14 FS|2026-09-02 vs Miami Marlins: 9 FS|2026-09-01 vs Miami Marlins: 2 FS</t>
         </is>
       </c>
       <c r="DF19" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06 vs New York Yankees: 0 FS|2026-09-05 vs New York Yankees: 2 FS|2026-09-04 vs New York Yankees: 0 FS|2026-09-02 @ Cincinnati Reds: 0 FS|2026-09-01 @ Cincinnati Reds: 8 FS|2026-08-31 @ Cincinnati Reds: 12 FS|2026-08-30 @ Tampa Bay Rays: 5 FS|2026-08-29 @ Tampa Bay Rays: 2 FS|2026-08-28 @ Tampa Bay Rays: 23 FS|2026-08-26 vs Pittsburgh Pirates: 19 FS</t>
+          <t>2026-09-05 vs Toronto Blue Jays: 5 FS|2026-09-04 vs Toronto Blue Jays: 0 FS|2026-09-03 vs Miami Marlins: 14 FS|2026-09-02 vs Miami Marlins: 9 FS|2026-09-01 vs Miami Marlins: 2 FS|2026-08-30 @ Cleveland Guardians: 7 FS|2026-08-29 @ Cleveland Guardians: 8 FS|2026-08-28 @ Cleveland Guardians: 6 FS|2026-08-27 @ Toronto Blue Jays: 42 FS|2026-08-26 @ Toronto Blue Jays: 0 FS</t>
         </is>
       </c>
       <c r="DG19" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06 vs New York Yankees: 0 FS|2026-09-05 vs New York Yankees: 2 FS|2026-09-04 vs New York Yankees: 0 FS|2026-09-02 @ Cincinnati Reds: 0 FS|2026-09-01 @ Cincinnati Reds: 8 FS|2026-08-31 @ Cincinnati Reds: 12 FS|2026-08-30 @ Tampa Bay Rays: 5 FS|2026-08-29 @ Tampa Bay Rays: 2 FS|2026-08-28 @ Tampa Bay Rays: 23 FS|2026-08-26 vs Pittsburgh Pirates: 19 FS|2026-08-25 vs Pittsburgh Pirates: 0 FS|2026-08-24 vs Pittsburgh Pirates: 0 FS|2026-08-23 vs Minnesota Twins: 14 FS|2026-08-22 vs Minnesota Twins: 21 FS|2026-08-21 vs Minnesota Twins: 0 FS</t>
+          <t>2026-09-05 vs Toronto Blue Jays: 5 FS|2026-09-04 vs Toronto Blue Jays: 0 FS|2026-09-03 vs Miami Marlins: 14 FS|2026-09-02 vs Miami Marlins: 9 FS|2026-09-01 vs Miami Marlins: 2 FS|2026-08-30 @ Cleveland Guardians: 7 FS|2026-08-29 @ Cleveland Guardians: 8 FS|2026-08-28 @ Cleveland Guardians: 6 FS|2026-08-27 @ Toronto Blue Jays: 42 FS|2026-08-26 @ Toronto Blue Jays: 0 FS|2026-08-22 vs Detroit Tigers: 7 FS|2026-08-21 vs Detroit Tigers: 0 FS|2026-08-19 vs Athletics: 5 FS|2026-08-18 vs Athletics: 10 FS|2026-08-17 vs Athletics: 15 FS</t>
         </is>
       </c>
       <c r="DH19" s="3" t="n">
@@ -17274,7 +17274,7 @@
         <v>30</v>
       </c>
       <c r="DJ19" s="3" t="n">
-        <v>8.17</v>
+        <v>10.4</v>
       </c>
       <c r="DK19" s="3" t="n">
         <v>7</v>
@@ -17285,54 +17285,54 @@
         </is>
       </c>
       <c r="DM19" s="3" t="n">
-        <v>3.86</v>
+        <v>6.43</v>
       </c>
       <c r="DN19" s="3" t="n">
-        <v>7.57</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="DO19" s="3" t="n">
-        <v>0.226</v>
+        <v>0.34</v>
       </c>
       <c r="DP19" s="4" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Hot</t>
         </is>
       </c>
       <c r="DQ19" s="3" t="n">
-        <v>8.17</v>
+        <v>10.4</v>
       </c>
       <c r="DR19" s="3" t="n">
-        <v>1.767</v>
+        <v>2.091</v>
       </c>
       <c r="DS19" s="3" t="n">
-        <v>0.2</v>
+        <v>0.3273</v>
       </c>
       <c r="DT19" s="3" t="n">
-        <v>0.1</v>
+        <v>0.1273</v>
       </c>
       <c r="DU19" s="3" t="n">
-        <v>0.05</v>
+        <v>0.0182</v>
       </c>
       <c r="DV19" s="3" t="n">
-        <v>0.0833</v>
+        <v>0.0182</v>
       </c>
       <c r="DW19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="DX19" s="3" t="n">
-        <v>8.26</v>
+        <v>8.48</v>
       </c>
       <c r="DY19" s="3" t="n">
-        <v>8.220000000000001</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="DZ19" s="3" t="n">
-        <v>7.89</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="EA19" s="3" t="n">
-        <v>7.14</v>
+        <v>7.77</v>
       </c>
       <c r="EB19" s="3" t="n">
-        <v>7.2</v>
+        <v>8.09</v>
       </c>
       <c r="EC19" s="3" t="n">
         <v>28</v>
@@ -17350,13 +17350,13 @@
         <v>20</v>
       </c>
       <c r="EH19" s="3" t="n">
-        <v>4.132</v>
+        <v>4.115</v>
       </c>
       <c r="EI19" s="3" t="n">
-        <v>0.0939</v>
+        <v>0.1539</v>
       </c>
       <c r="EJ19" s="3" t="n">
-        <v>0.08409999999999999</v>
+        <v>0.1935</v>
       </c>
       <c r="EK19" s="4" t="inlineStr">
         <is>
@@ -17370,28 +17370,28 @@
         <v>20</v>
       </c>
       <c r="EN19" s="3" t="n">
-        <v>0.88</v>
+        <v>1.072</v>
       </c>
       <c r="EO19" s="3" t="n">
-        <v>322</v>
+        <v>242</v>
       </c>
       <c r="EP19" s="3" t="n">
-        <v>84.78</v>
+        <v>86.67</v>
       </c>
       <c r="EQ19" s="3" t="n">
-        <v>27.33</v>
+        <v>35.95</v>
       </c>
       <c r="ER19" s="3" t="n">
-        <v>3.73</v>
+        <v>0.83</v>
       </c>
       <c r="ES19" s="3" t="n">
-        <v>34.47</v>
+        <v>26.45</v>
       </c>
       <c r="ET19" s="3" t="n">
-        <v>0.487</v>
+        <v>0.422</v>
       </c>
       <c r="EU19" s="3" t="n">
-        <v>1.0378</v>
+        <v>1.0146</v>
       </c>
       <c r="EV19" s="3" t="n">
         <v>1</v>
@@ -17403,74 +17403,74 @@
         <v>1</v>
       </c>
       <c r="EY19" s="3" t="n">
-        <v>1.0644</v>
+        <v>1</v>
       </c>
       <c r="EZ19" s="3" t="n">
-        <v>581</v>
+        <v>0</v>
       </c>
       <c r="FA19" s="4" t="inlineStr">
         <is>
-          <t>Statcast</t>
+          <t>Fallback</t>
         </is>
       </c>
       <c r="FB19" s="3" t="n">
-        <v>1.14</v>
+        <v>1</v>
       </c>
       <c r="FC19" s="3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="FD19" s="4" t="inlineStr">
         <is>
-          <t>Statcast</t>
+          <t>Fallback</t>
         </is>
       </c>
       <c r="FE19" s="3" t="n">
-        <v>322</v>
+        <v>242</v>
       </c>
       <c r="FF19" s="3" t="n">
-        <v>84.78</v>
+        <v>86.67</v>
       </c>
       <c r="FG19" s="3" t="n">
         <v>12</v>
       </c>
       <c r="FH19" s="3" t="n">
-        <v>20.36</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="FI19" s="3" t="n">
-        <v>29.41</v>
+        <v>32.1</v>
       </c>
       <c r="FJ19" s="3" t="n">
-        <v>14.9</v>
+        <v>12.8</v>
       </c>
       <c r="FK19" s="3" t="n">
-        <v>64.59999999999999</v>
+        <v>54.1</v>
       </c>
       <c r="FL19" s="3" t="n">
-        <v>20.5</v>
+        <v>33.1</v>
       </c>
       <c r="FM19" s="3" t="n">
-        <v>0.9895</v>
+        <v>1.0307</v>
       </c>
       <c r="FN19" s="3" t="n">
-        <v>0.9947</v>
+        <v>1.0051</v>
       </c>
       <c r="FO19" s="3" t="n">
-        <v>1.0067</v>
+        <v>1.0498</v>
       </c>
       <c r="FP19" s="3" t="n">
-        <v>1.0499</v>
+        <v>1.0101</v>
       </c>
       <c r="FQ19" s="3" t="n">
-        <v>0.9288999999999999</v>
+        <v>1.0655</v>
       </c>
       <c r="FR19" s="3" t="n">
-        <v>0.9699</v>
+        <v>0.9785</v>
       </c>
       <c r="FS19" s="3" t="n">
-        <v>5.66</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="FT19" s="3" t="n">
-        <v>-2.51</v>
+        <v>-1.79</v>
       </c>
       <c r="FU19" s="4" t="inlineStr">
         <is>
@@ -17515,52 +17515,52 @@
         <v>27</v>
       </c>
       <c r="GG19" s="3" t="n">
-        <v>1.3</v>
+        <v>1.0517</v>
       </c>
       <c r="GH19" s="3" t="n">
         <v>27</v>
       </c>
       <c r="GI19" s="3" t="n">
-        <v>0.9855</v>
+        <v>1</v>
       </c>
       <c r="GJ19" s="3" t="n">
-        <v>0.139</v>
+        <v>0.1535</v>
       </c>
       <c r="GK19" s="3" t="n">
-        <v>0.0432</v>
+        <v>0.0659</v>
       </c>
       <c r="GL19" s="3" t="n">
-        <v>0.005</v>
+        <v>0.0038</v>
       </c>
       <c r="GM19" s="3" t="n">
-        <v>0.0474</v>
+        <v>0.0407</v>
       </c>
       <c r="GN19" s="3" t="n">
-        <v>0.0902</v>
+        <v>0.066</v>
       </c>
       <c r="GO19" s="3" t="n">
-        <v>0.0128</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="GP19" s="3" t="n">
-        <v>0.2333</v>
+        <v>0.2378</v>
       </c>
       <c r="GQ19" s="3" t="n">
-        <v>0.3195</v>
+        <v>0.518</v>
       </c>
       <c r="GR19" s="3" t="n">
-        <v>0.375</v>
+        <v>0.2302</v>
       </c>
       <c r="GS19" s="3" t="n">
-        <v>0.3055</v>
+        <v>0.2518</v>
       </c>
       <c r="GT19" s="3" t="n">
-        <v>0.107</v>
+        <v>0.1348</v>
       </c>
       <c r="GU19" s="3" t="n">
-        <v>0.1087</v>
+        <v>0.1689</v>
       </c>
       <c r="GV19" s="3" t="n">
-        <v>0.0201</v>
+        <v>0.0118</v>
       </c>
       <c r="GW19" s="3" t="n">
         <v>1</v>
@@ -17571,22 +17571,22 @@
         </is>
       </c>
       <c r="GY19" s="3" t="n">
-        <v>7.03</v>
+        <v>8.35</v>
       </c>
       <c r="GZ19" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0</v>
       </c>
       <c r="HA19" s="3" t="n">
-        <v>9.75</v>
+        <v>10.04</v>
       </c>
       <c r="HB19" s="3" t="n">
-        <v>17.1</v>
+        <v>19.1</v>
       </c>
       <c r="HC19" s="3" t="n">
-        <v>3.72</v>
+        <v>3.71</v>
       </c>
       <c r="HD19" s="3" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="HE19" s="4" t="inlineStr">
         <is>
@@ -17594,85 +17594,85 @@
         </is>
       </c>
       <c r="HF19" s="3" t="n">
-        <v>63.1</v>
+        <v>55</v>
       </c>
       <c r="HG19" s="3" t="n">
-        <v>63.1</v>
+        <v>55</v>
       </c>
       <c r="HH19" s="3" t="n">
-        <v>54.9</v>
+        <v>52.8</v>
       </c>
       <c r="HI19" s="3" t="n">
-        <v>54.9</v>
+        <v>52.8</v>
       </c>
       <c r="HJ19" s="3" t="n">
-        <v>51.5</v>
+        <v>43.8</v>
       </c>
       <c r="HK19" s="3" t="n">
-        <v>51.5</v>
+        <v>43.8</v>
       </c>
       <c r="HL19" s="3" t="n">
-        <v>41.6</v>
+        <v>43.8</v>
       </c>
       <c r="HM19" s="3" t="n">
-        <v>41.6</v>
+        <v>40.8</v>
       </c>
       <c r="HN19" s="3" t="n">
-        <v>39.3</v>
+        <v>40.8</v>
       </c>
       <c r="HO19" s="3" t="n">
-        <v>33.6</v>
+        <v>34.9</v>
       </c>
       <c r="HP19" s="3" t="n">
-        <v>33.6</v>
+        <v>34.9</v>
       </c>
       <c r="HQ19" s="3" t="n">
-        <v>30.4</v>
+        <v>30.9</v>
       </c>
       <c r="HR19" s="3" t="n">
-        <v>30.4</v>
+        <v>30.9</v>
       </c>
       <c r="HS19" s="3" t="n">
-        <v>27.1</v>
+        <v>28</v>
       </c>
       <c r="HT19" s="3" t="n">
-        <v>27.1</v>
+        <v>28</v>
       </c>
       <c r="HU19" s="3" t="n">
-        <v>24.4</v>
+        <v>28</v>
       </c>
       <c r="HV19" s="3" t="n">
-        <v>24.4</v>
+        <v>24.2</v>
       </c>
       <c r="HW19" s="3" t="n">
-        <v>22.8</v>
+        <v>24.2</v>
       </c>
       <c r="HX19" s="3" t="n">
-        <v>22.8</v>
+        <v>22.6</v>
       </c>
       <c r="HY19" s="3" t="n">
-        <v>21</v>
+        <v>22.6</v>
       </c>
       <c r="HZ19" s="3" t="n">
-        <v>21</v>
+        <v>20.1</v>
       </c>
       <c r="IA19" s="3" t="n">
-        <v>20</v>
+        <v>20.1</v>
       </c>
       <c r="IB19" s="3" t="n">
-        <v>16.5</v>
+        <v>18.8</v>
       </c>
       <c r="IC19" s="3" t="n">
-        <v>16.5</v>
+        <v>18.8</v>
       </c>
       <c r="ID19" s="3" t="n">
-        <v>15.7</v>
+        <v>18.8</v>
       </c>
       <c r="IE19" s="3" t="n">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="IF19" s="3" t="n">
-        <v>13</v>
+        <v>15.8</v>
       </c>
       <c r="IG19" s="3" t="n">
         <v>0</v>
@@ -17775,22 +17775,22 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Jac Caglianone</t>
+          <t>Jackson Merrill</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>KC</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>ARI @ KC</t>
+          <t>WSH @ SD</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -17800,170 +17800,170 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="J20" s="3" t="n">
-        <v>8.42</v>
+        <v>7.79</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>6.92</v>
+        <v>6.84</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>6.92</v>
+        <v>6.84</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>4.37</v>
+        <v>5.15</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>9.949999999999999</v>
+        <v>7.58</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>8.68</v>
+        <v>7.03</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>7.66</v>
+        <v>7.64</v>
       </c>
       <c r="Q20" s="3" t="n">
-        <v>8.35</v>
+        <v>7.03</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>1.133</v>
+        <v>0.921</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>7.1</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>8.67</v>
+        <v>7.07</v>
       </c>
       <c r="V20" s="4" t="inlineStr">
         <is>
-          <t>5|0|14|9|2</t>
+          <t>0|2|0|0|8</t>
         </is>
       </c>
       <c r="W20" s="4" t="inlineStr">
         <is>
-          <t>5|0|14|9|2|7|8|6|42|0</t>
+          <t>0|2|0|0|8|12|5|2|23|19</t>
         </is>
       </c>
       <c r="X20" s="4" t="inlineStr">
         <is>
-          <t>5|0|14|9|2|7|8|6|42|0|7|0|5|10|15</t>
-        </is>
-      </c>
-      <c r="Y20" s="6" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="Z20" s="7" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="AA20" s="7" t="n">
-        <v>52.3</v>
+          <t>0|2|0|0|8|12|5|2|23|19|0|0|14|21|0</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="Z20" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="AA20" s="6" t="n">
+        <v>54.6</v>
       </c>
       <c r="AB20" s="7" t="n">
-        <v>50.5</v>
+        <v>53.6</v>
       </c>
       <c r="AC20" s="7" t="n">
-        <v>45.5</v>
+        <v>51.9</v>
       </c>
       <c r="AD20" s="7" t="n">
-        <v>43.8</v>
+        <v>48</v>
       </c>
       <c r="AE20" s="7" t="n">
-        <v>43.8</v>
+        <v>42.8</v>
       </c>
       <c r="AF20" s="7" t="n">
-        <v>40.8</v>
-      </c>
-      <c r="AG20" s="7" t="n">
-        <v>40.6</v>
+        <v>41.2</v>
+      </c>
+      <c r="AG20" s="8" t="n">
+        <v>39.8</v>
       </c>
       <c r="AH20" s="8" t="n">
-        <v>34.6</v>
+        <v>34</v>
       </c>
       <c r="AI20" s="8" t="n">
-        <v>34.6</v>
+        <v>34</v>
       </c>
       <c r="AJ20" s="8" t="n">
-        <v>31.2</v>
+        <v>30.6</v>
       </c>
       <c r="AK20" s="8" t="n">
-        <v>31.2</v>
+        <v>30.6</v>
       </c>
       <c r="AL20" s="8" t="n">
-        <v>28.6</v>
+        <v>28.2</v>
       </c>
       <c r="AM20" s="8" t="n">
-        <v>28.5</v>
+        <v>28.1</v>
       </c>
       <c r="AN20" s="8" t="n">
-        <v>27.2</v>
+        <v>24.8</v>
       </c>
       <c r="AO20" s="8" t="n">
         <v>24.8</v>
       </c>
       <c r="AP20" s="8" t="n">
-        <v>23.5</v>
+        <v>22.7</v>
       </c>
       <c r="AQ20" s="8" t="n">
-        <v>23.3</v>
+        <v>22.7</v>
       </c>
       <c r="AR20" s="8" t="n">
-        <v>22.5</v>
+        <v>20.8</v>
       </c>
       <c r="AS20" s="8" t="n">
-        <v>20.9</v>
+        <v>20.8</v>
       </c>
       <c r="AT20" s="8" t="n">
-        <v>20.1</v>
+        <v>20</v>
       </c>
       <c r="AU20" s="8" t="n">
-        <v>19.6</v>
+        <v>18.2</v>
       </c>
       <c r="AV20" s="8" t="n">
-        <v>17.9</v>
+        <v>16.1</v>
       </c>
       <c r="AW20" s="8" t="n">
-        <v>17.9</v>
+        <v>16.1</v>
       </c>
       <c r="AX20" s="8" t="n">
-        <v>16.3</v>
+        <v>16.1</v>
       </c>
       <c r="AY20" s="8" t="n">
-        <v>16.3</v>
+        <v>13.5</v>
       </c>
       <c r="AZ20" s="3" t="n">
-        <v>188.47</v>
+        <v>188.33</v>
       </c>
       <c r="BA20" s="4" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="BB20" s="10" t="inlineStr">
-        <is>
-          <t>LESS 7.5 | 65.4% | Edge +0.6</t>
+      <c r="BB20" s="9" t="inlineStr">
+        <is>
+          <t>MORE 3.0 | 59.0% | Edge +3.8</t>
         </is>
       </c>
       <c r="BC20" s="4" t="inlineStr">
         <is>
-          <t>LESS</t>
+          <t>MORE</t>
         </is>
       </c>
       <c r="BD20" s="3" t="n">
-        <v>7.5</v>
+        <v>3</v>
       </c>
       <c r="BE20" s="3" t="n">
-        <v>65.40000000000001</v>
+        <v>59</v>
       </c>
       <c r="BF20" s="3" t="n">
-        <v>0.58</v>
+        <v>3.84</v>
       </c>
       <c r="BG20" s="3" t="n">
-        <v>30.8</v>
+        <v>18</v>
       </c>
       <c r="BH20" s="4" t="inlineStr">
         <is>
@@ -17971,7 +17971,7 @@
         </is>
       </c>
       <c r="BI20" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BJ20" s="4" t="inlineStr">
         <is>
@@ -17980,24 +17980,24 @@
       </c>
       <c r="BK20" s="4" t="n"/>
       <c r="BL20" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BM20" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BN20" s="4" t="inlineStr">
         <is>
-          <t>3-3-3-3-3-3</t>
+          <t>5-5-5-3-5-5-5</t>
         </is>
       </c>
       <c r="BO20" s="3" t="n">
-        <v>100</v>
+        <v>85.7</v>
       </c>
       <c r="BP20" s="3" t="n">
         <v>97</v>
       </c>
       <c r="BQ20" s="3" t="n">
-        <v>4.12</v>
+        <v>4.13</v>
       </c>
       <c r="BR20" s="4" t="inlineStr">
         <is>
@@ -18005,14 +18005,14 @@
         </is>
       </c>
       <c r="BS20" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="BT20" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="BU20" s="4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Jake Irvin</t>
         </is>
       </c>
       <c r="BV20" s="4" t="inlineStr">
@@ -18021,124 +18021,124 @@
         </is>
       </c>
       <c r="BW20" s="3" t="n">
-        <v>4.2</v>
+        <v>5.57</v>
       </c>
       <c r="BX20" s="3" t="n">
-        <v>1.25</v>
+        <v>1.4</v>
       </c>
       <c r="BY20" s="3" t="n">
-        <v>0.224</v>
+        <v>0.2105</v>
       </c>
       <c r="BZ20" s="3" t="n">
-        <v>0.03</v>
+        <v>0.0395</v>
       </c>
       <c r="CA20" s="3" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.1053</v>
       </c>
       <c r="CB20" s="3" t="n">
-        <v>4.13</v>
+        <v>4.72</v>
       </c>
       <c r="CC20" s="3" t="n">
-        <v>1.28</v>
+        <v>1.39</v>
       </c>
       <c r="CD20" s="3" t="n">
-        <v>0.2235</v>
+        <v>0.2243</v>
       </c>
       <c r="CE20" s="3" t="n">
-        <v>0.03</v>
+        <v>0.0351</v>
       </c>
       <c r="CF20" s="4" t="inlineStr">
         <is>
-          <t>Kauffman Stadium</t>
+          <t>Petco Park</t>
         </is>
       </c>
       <c r="CG20" s="3" t="n">
-        <v>1.072</v>
+        <v>0.88</v>
       </c>
       <c r="CH20" s="3" t="n">
-        <v>1.03</v>
+        <v>1.065</v>
       </c>
       <c r="CI20" s="3" t="n">
-        <v>89.59999999999999</v>
+        <v>94.2</v>
       </c>
       <c r="CJ20" s="3" t="n">
-        <v>8.4</v>
+        <v>11.9</v>
       </c>
       <c r="CK20" s="3" t="n">
-        <v>158</v>
+        <v>322</v>
       </c>
       <c r="CL20" s="3" t="n">
         <v>2</v>
       </c>
       <c r="CM20" s="4" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>hot, light wind</t>
         </is>
       </c>
       <c r="CN20" s="3" t="n">
-        <v>510</v>
+        <v>587</v>
       </c>
       <c r="CO20" s="3" t="n">
-        <v>474</v>
+        <v>540</v>
       </c>
       <c r="CP20" s="3" t="n">
-        <v>0.283</v>
+        <v>0.237</v>
       </c>
       <c r="CQ20" s="3" t="n">
-        <v>0.331</v>
+        <v>0.29</v>
       </c>
       <c r="CR20" s="3" t="n">
-        <v>0.494</v>
+        <v>0.411</v>
       </c>
       <c r="CS20" s="3" t="n">
-        <v>0.825</v>
+        <v>0.701</v>
       </c>
       <c r="CT20" s="3" t="n">
-        <v>355</v>
+        <v>421</v>
       </c>
       <c r="CU20" s="3" t="n">
-        <v>0.864</v>
+        <v>0.699</v>
       </c>
       <c r="CV20" s="3" t="n">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="CW20" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="CX20" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CY20" s="3" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="CZ20" s="3" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="DA20" s="3" t="n">
         <v>70</v>
       </c>
       <c r="DB20" s="3" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="DC20" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="DD20" s="3" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="DE20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05 vs Toronto Blue Jays: 5 FS|2026-09-04 vs Toronto Blue Jays: 0 FS|2026-09-03 vs Miami Marlins: 14 FS|2026-09-02 vs Miami Marlins: 9 FS|2026-09-01 vs Miami Marlins: 2 FS</t>
+          <t>2026-09-06 vs New York Yankees: 0 FS|2026-09-05 vs New York Yankees: 2 FS|2026-09-04 vs New York Yankees: 0 FS|2026-09-02 @ Cincinnati Reds: 0 FS|2026-09-01 @ Cincinnati Reds: 8 FS</t>
         </is>
       </c>
       <c r="DF20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05 vs Toronto Blue Jays: 5 FS|2026-09-04 vs Toronto Blue Jays: 0 FS|2026-09-03 vs Miami Marlins: 14 FS|2026-09-02 vs Miami Marlins: 9 FS|2026-09-01 vs Miami Marlins: 2 FS|2026-08-30 @ Cleveland Guardians: 7 FS|2026-08-29 @ Cleveland Guardians: 8 FS|2026-08-28 @ Cleveland Guardians: 6 FS|2026-08-27 @ Toronto Blue Jays: 42 FS|2026-08-26 @ Toronto Blue Jays: 0 FS</t>
+          <t>2026-09-06 vs New York Yankees: 0 FS|2026-09-05 vs New York Yankees: 2 FS|2026-09-04 vs New York Yankees: 0 FS|2026-09-02 @ Cincinnati Reds: 0 FS|2026-09-01 @ Cincinnati Reds: 8 FS|2026-08-31 @ Cincinnati Reds: 12 FS|2026-08-30 @ Tampa Bay Rays: 5 FS|2026-08-29 @ Tampa Bay Rays: 2 FS|2026-08-28 @ Tampa Bay Rays: 23 FS|2026-08-26 vs Pittsburgh Pirates: 19 FS</t>
         </is>
       </c>
       <c r="DG20" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05 vs Toronto Blue Jays: 5 FS|2026-09-04 vs Toronto Blue Jays: 0 FS|2026-09-03 vs Miami Marlins: 14 FS|2026-09-02 vs Miami Marlins: 9 FS|2026-09-01 vs Miami Marlins: 2 FS|2026-08-30 @ Cleveland Guardians: 7 FS|2026-08-29 @ Cleveland Guardians: 8 FS|2026-08-28 @ Cleveland Guardians: 6 FS|2026-08-27 @ Toronto Blue Jays: 42 FS|2026-08-26 @ Toronto Blue Jays: 0 FS|2026-08-22 vs Detroit Tigers: 7 FS|2026-08-21 vs Detroit Tigers: 0 FS|2026-08-19 vs Athletics: 5 FS|2026-08-18 vs Athletics: 10 FS|2026-08-17 vs Athletics: 15 FS</t>
+          <t>2026-09-06 vs New York Yankees: 0 FS|2026-09-05 vs New York Yankees: 2 FS|2026-09-04 vs New York Yankees: 0 FS|2026-09-02 @ Cincinnati Reds: 0 FS|2026-09-01 @ Cincinnati Reds: 8 FS|2026-08-31 @ Cincinnati Reds: 12 FS|2026-08-30 @ Tampa Bay Rays: 5 FS|2026-08-29 @ Tampa Bay Rays: 2 FS|2026-08-28 @ Tampa Bay Rays: 23 FS|2026-08-26 vs Pittsburgh Pirates: 19 FS|2026-08-25 vs Pittsburgh Pirates: 0 FS|2026-08-24 vs Pittsburgh Pirates: 0 FS|2026-08-23 vs Minnesota Twins: 14 FS|2026-08-22 vs Minnesota Twins: 21 FS|2026-08-21 vs Minnesota Twins: 0 FS</t>
         </is>
       </c>
       <c r="DH20" s="3" t="n">
@@ -18148,7 +18148,7 @@
         <v>30</v>
       </c>
       <c r="DJ20" s="3" t="n">
-        <v>10.4</v>
+        <v>8.17</v>
       </c>
       <c r="DK20" s="3" t="n">
         <v>7</v>
@@ -18159,54 +18159,54 @@
         </is>
       </c>
       <c r="DM20" s="3" t="n">
-        <v>6.43</v>
+        <v>3.86</v>
       </c>
       <c r="DN20" s="3" t="n">
-        <v>8.210000000000001</v>
+        <v>7.57</v>
       </c>
       <c r="DO20" s="3" t="n">
-        <v>0.34</v>
+        <v>0.226</v>
       </c>
       <c r="DP20" s="4" t="inlineStr">
         <is>
-          <t>Hot</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="DQ20" s="3" t="n">
-        <v>10.4</v>
+        <v>8.17</v>
       </c>
       <c r="DR20" s="3" t="n">
-        <v>2.091</v>
+        <v>1.767</v>
       </c>
       <c r="DS20" s="3" t="n">
-        <v>0.3273</v>
+        <v>0.2</v>
       </c>
       <c r="DT20" s="3" t="n">
-        <v>0.1273</v>
+        <v>0.1</v>
       </c>
       <c r="DU20" s="3" t="n">
-        <v>0.0182</v>
+        <v>0.05</v>
       </c>
       <c r="DV20" s="3" t="n">
-        <v>0.0182</v>
+        <v>0.0833</v>
       </c>
       <c r="DW20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="DX20" s="3" t="n">
-        <v>8.48</v>
+        <v>8.26</v>
       </c>
       <c r="DY20" s="3" t="n">
-        <v>9.529999999999999</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="DZ20" s="3" t="n">
-        <v>8.279999999999999</v>
+        <v>7.89</v>
       </c>
       <c r="EA20" s="3" t="n">
-        <v>7.77</v>
+        <v>7.14</v>
       </c>
       <c r="EB20" s="3" t="n">
-        <v>8.09</v>
+        <v>7.2</v>
       </c>
       <c r="EC20" s="3" t="n">
         <v>28</v>
@@ -18224,13 +18224,13 @@
         <v>20</v>
       </c>
       <c r="EH20" s="3" t="n">
-        <v>4.115</v>
+        <v>4.132</v>
       </c>
       <c r="EI20" s="3" t="n">
-        <v>0.1539</v>
+        <v>0.0939</v>
       </c>
       <c r="EJ20" s="3" t="n">
-        <v>0.1935</v>
+        <v>0.08409999999999999</v>
       </c>
       <c r="EK20" s="4" t="inlineStr">
         <is>
@@ -18244,28 +18244,28 @@
         <v>20</v>
       </c>
       <c r="EN20" s="3" t="n">
-        <v>1.072</v>
+        <v>0.88</v>
       </c>
       <c r="EO20" s="3" t="n">
-        <v>242</v>
+        <v>322</v>
       </c>
       <c r="EP20" s="3" t="n">
-        <v>86.67</v>
+        <v>84.78</v>
       </c>
       <c r="EQ20" s="3" t="n">
-        <v>35.95</v>
+        <v>27.33</v>
       </c>
       <c r="ER20" s="3" t="n">
-        <v>0.83</v>
+        <v>3.73</v>
       </c>
       <c r="ES20" s="3" t="n">
-        <v>26.45</v>
+        <v>34.47</v>
       </c>
       <c r="ET20" s="3" t="n">
-        <v>0.422</v>
+        <v>0.487</v>
       </c>
       <c r="EU20" s="3" t="n">
-        <v>1.0146</v>
+        <v>1.0378</v>
       </c>
       <c r="EV20" s="3" t="n">
         <v>1</v>
@@ -18277,74 +18277,74 @@
         <v>1</v>
       </c>
       <c r="EY20" s="3" t="n">
-        <v>1</v>
+        <v>1.0644</v>
       </c>
       <c r="EZ20" s="3" t="n">
-        <v>0</v>
+        <v>581</v>
       </c>
       <c r="FA20" s="4" t="inlineStr">
         <is>
-          <t>Fallback</t>
+          <t>Statcast</t>
         </is>
       </c>
       <c r="FB20" s="3" t="n">
-        <v>1</v>
+        <v>1.14</v>
       </c>
       <c r="FC20" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="FD20" s="4" t="inlineStr">
         <is>
-          <t>Fallback</t>
+          <t>Statcast</t>
         </is>
       </c>
       <c r="FE20" s="3" t="n">
-        <v>242</v>
+        <v>322</v>
       </c>
       <c r="FF20" s="3" t="n">
-        <v>86.67</v>
+        <v>84.78</v>
       </c>
       <c r="FG20" s="3" t="n">
         <v>12</v>
       </c>
       <c r="FH20" s="3" t="n">
-        <v>9.199999999999999</v>
+        <v>20.36</v>
       </c>
       <c r="FI20" s="3" t="n">
-        <v>32.1</v>
+        <v>29.41</v>
       </c>
       <c r="FJ20" s="3" t="n">
-        <v>12.8</v>
+        <v>14.9</v>
       </c>
       <c r="FK20" s="3" t="n">
-        <v>54.1</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="FL20" s="3" t="n">
-        <v>33.1</v>
+        <v>20.5</v>
       </c>
       <c r="FM20" s="3" t="n">
-        <v>1.0307</v>
+        <v>0.9893</v>
       </c>
       <c r="FN20" s="3" t="n">
-        <v>1.0051</v>
+        <v>0.9947</v>
       </c>
       <c r="FO20" s="3" t="n">
-        <v>1.0498</v>
+        <v>1.0065</v>
       </c>
       <c r="FP20" s="3" t="n">
-        <v>1.0101</v>
+        <v>1.0499</v>
       </c>
       <c r="FQ20" s="3" t="n">
-        <v>1.0655</v>
+        <v>0.9287</v>
       </c>
       <c r="FR20" s="3" t="n">
-        <v>0.9785</v>
+        <v>0.9699</v>
       </c>
       <c r="FS20" s="3" t="n">
-        <v>8.609999999999999</v>
+        <v>5.66</v>
       </c>
       <c r="FT20" s="3" t="n">
-        <v>-1.79</v>
+        <v>-2.51</v>
       </c>
       <c r="FU20" s="4" t="inlineStr">
         <is>
@@ -18389,52 +18389,52 @@
         <v>27</v>
       </c>
       <c r="GG20" s="3" t="n">
-        <v>1.0517</v>
+        <v>1.3</v>
       </c>
       <c r="GH20" s="3" t="n">
         <v>27</v>
       </c>
       <c r="GI20" s="3" t="n">
-        <v>1</v>
+        <v>0.9855</v>
       </c>
       <c r="GJ20" s="3" t="n">
-        <v>0.1535</v>
+        <v>0.139</v>
       </c>
       <c r="GK20" s="3" t="n">
-        <v>0.0659</v>
+        <v>0.0432</v>
       </c>
       <c r="GL20" s="3" t="n">
-        <v>0.0038</v>
+        <v>0.005</v>
       </c>
       <c r="GM20" s="3" t="n">
-        <v>0.0407</v>
+        <v>0.0474</v>
       </c>
       <c r="GN20" s="3" t="n">
-        <v>0.066</v>
+        <v>0.0902</v>
       </c>
       <c r="GO20" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0128</v>
       </c>
       <c r="GP20" s="3" t="n">
-        <v>0.2378</v>
+        <v>0.2333</v>
       </c>
       <c r="GQ20" s="3" t="n">
-        <v>0.518</v>
+        <v>0.3195</v>
       </c>
       <c r="GR20" s="3" t="n">
-        <v>0.2302</v>
+        <v>0.375</v>
       </c>
       <c r="GS20" s="3" t="n">
-        <v>0.2518</v>
+        <v>0.3055</v>
       </c>
       <c r="GT20" s="3" t="n">
-        <v>0.1348</v>
+        <v>0.107</v>
       </c>
       <c r="GU20" s="3" t="n">
-        <v>0.1689</v>
+        <v>0.1087</v>
       </c>
       <c r="GV20" s="3" t="n">
-        <v>0.0118</v>
+        <v>0.0201</v>
       </c>
       <c r="GW20" s="3" t="n">
         <v>1</v>
@@ -18445,22 +18445,22 @@
         </is>
       </c>
       <c r="GY20" s="3" t="n">
-        <v>8.35</v>
+        <v>7.03</v>
       </c>
       <c r="GZ20" s="3" t="n">
-        <v>0</v>
+        <v>0.54</v>
       </c>
       <c r="HA20" s="3" t="n">
-        <v>10.04</v>
+        <v>9.75</v>
       </c>
       <c r="HB20" s="3" t="n">
-        <v>19.1</v>
+        <v>17.12</v>
       </c>
       <c r="HC20" s="3" t="n">
         <v>3.71</v>
       </c>
       <c r="HD20" s="3" t="n">
-        <v>14</v>
+        <v>11.1</v>
       </c>
       <c r="HE20" s="4" t="inlineStr">
         <is>
@@ -18468,85 +18468,85 @@
         </is>
       </c>
       <c r="HF20" s="3" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="HG20" s="3" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="HH20" s="3" t="n">
-        <v>52.8</v>
+        <v>54.8</v>
       </c>
       <c r="HI20" s="3" t="n">
-        <v>52.8</v>
+        <v>54.8</v>
       </c>
       <c r="HJ20" s="3" t="n">
-        <v>43.8</v>
+        <v>51.4</v>
       </c>
       <c r="HK20" s="3" t="n">
-        <v>43.8</v>
+        <v>51.4</v>
       </c>
       <c r="HL20" s="3" t="n">
-        <v>43.8</v>
+        <v>41.5</v>
       </c>
       <c r="HM20" s="3" t="n">
-        <v>40.8</v>
+        <v>41.5</v>
       </c>
       <c r="HN20" s="3" t="n">
-        <v>40.8</v>
+        <v>39.2</v>
       </c>
       <c r="HO20" s="3" t="n">
-        <v>34.9</v>
+        <v>33.6</v>
       </c>
       <c r="HP20" s="3" t="n">
-        <v>34.9</v>
+        <v>33.6</v>
       </c>
       <c r="HQ20" s="3" t="n">
-        <v>30.9</v>
+        <v>30.3</v>
       </c>
       <c r="HR20" s="3" t="n">
-        <v>30.9</v>
+        <v>30.3</v>
       </c>
       <c r="HS20" s="3" t="n">
-        <v>28</v>
+        <v>27.1</v>
       </c>
       <c r="HT20" s="3" t="n">
-        <v>28</v>
+        <v>27.1</v>
       </c>
       <c r="HU20" s="3" t="n">
-        <v>28</v>
+        <v>24.3</v>
       </c>
       <c r="HV20" s="3" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="HW20" s="3" t="n">
-        <v>24.2</v>
+        <v>22.7</v>
       </c>
       <c r="HX20" s="3" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="HY20" s="3" t="n">
-        <v>22.6</v>
+        <v>20.9</v>
       </c>
       <c r="HZ20" s="3" t="n">
-        <v>20.1</v>
+        <v>20.9</v>
       </c>
       <c r="IA20" s="3" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
       <c r="IB20" s="3" t="n">
-        <v>18.8</v>
+        <v>16.4</v>
       </c>
       <c r="IC20" s="3" t="n">
-        <v>18.8</v>
+        <v>16.4</v>
       </c>
       <c r="ID20" s="3" t="n">
-        <v>18.8</v>
+        <v>15.7</v>
       </c>
       <c r="IE20" s="3" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="IF20" s="3" t="n">
-        <v>15.8</v>
+        <v>12.9</v>
       </c>
       <c r="IG20" s="3" t="n">
         <v>0</v>
@@ -21303,10 +21303,10 @@
         <v>7.68</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>6.29</v>
+        <v>6.31</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>6.29</v>
+        <v>6.31</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>4.1</v>
@@ -21318,13 +21318,13 @@
         <v>6.62</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>6.91</v>
+        <v>6.93</v>
       </c>
       <c r="Q24" s="3" t="n">
         <v>6.62</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>0.958</v>
+        <v>0.955</v>
       </c>
       <c r="S24" s="3" t="n">
         <v>12.4</v>
@@ -21351,16 +21351,16 @@
         </is>
       </c>
       <c r="Y24" s="5" t="n">
-        <v>62.9</v>
+        <v>63</v>
       </c>
       <c r="Z24" s="5" t="n">
-        <v>58.7</v>
+        <v>58.8</v>
       </c>
       <c r="AA24" s="6" t="n">
-        <v>53.3</v>
+        <v>53.4</v>
       </c>
       <c r="AB24" s="7" t="n">
-        <v>53.3</v>
+        <v>53.4</v>
       </c>
       <c r="AC24" s="7" t="n">
         <v>48.7</v>
@@ -21372,7 +21372,7 @@
         <v>42.5</v>
       </c>
       <c r="AF24" s="7" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="AG24" s="8" t="n">
         <v>38.8</v>
@@ -21420,19 +21420,19 @@
         <v>16.8</v>
       </c>
       <c r="AV24" s="8" t="n">
-        <v>13.2</v>
+        <v>14</v>
       </c>
       <c r="AW24" s="8" t="n">
-        <v>13.2</v>
+        <v>14</v>
       </c>
       <c r="AX24" s="8" t="n">
-        <v>13.2</v>
+        <v>13.8</v>
       </c>
       <c r="AY24" s="8" t="n">
-        <v>13.2</v>
+        <v>13.5</v>
       </c>
       <c r="AZ24" s="3" t="n">
-        <v>183.49</v>
+        <v>183.77</v>
       </c>
       <c r="BA24" s="4" t="inlineStr">
         <is>
@@ -21441,7 +21441,7 @@
       </c>
       <c r="BB24" s="9" t="inlineStr">
         <is>
-          <t>MORE 3.0 | 58.7% | Edge +3.3</t>
+          <t>MORE 3.0 | 58.8% | Edge +3.3</t>
         </is>
       </c>
       <c r="BC24" s="4" t="inlineStr">
@@ -21453,13 +21453,13 @@
         <v>3</v>
       </c>
       <c r="BE24" s="3" t="n">
-        <v>58.7</v>
+        <v>58.8</v>
       </c>
       <c r="BF24" s="3" t="n">
-        <v>3.29</v>
+        <v>3.31</v>
       </c>
       <c r="BG24" s="3" t="n">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="BH24" s="4" t="inlineStr">
         <is>
@@ -21555,13 +21555,13 @@
         <v>1.065</v>
       </c>
       <c r="CI24" s="3" t="n">
-        <v>95.09999999999999</v>
+        <v>94.2</v>
       </c>
       <c r="CJ24" s="3" t="n">
-        <v>12.2</v>
+        <v>11.9</v>
       </c>
       <c r="CK24" s="3" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="CL24" s="3" t="n">
         <v>2</v>
@@ -21819,19 +21819,19 @@
         <v>15.9</v>
       </c>
       <c r="FM24" s="3" t="n">
-        <v>0.9895</v>
+        <v>0.9893</v>
       </c>
       <c r="FN24" s="3" t="n">
         <v>0.9921</v>
       </c>
       <c r="FO24" s="3" t="n">
-        <v>0.9974</v>
+        <v>0.9972</v>
       </c>
       <c r="FP24" s="3" t="n">
         <v>1.0445</v>
       </c>
       <c r="FQ24" s="3" t="n">
-        <v>0.9134</v>
+        <v>0.9133</v>
       </c>
       <c r="FR24" s="3" t="n">
         <v>1.0272</v>
@@ -21891,7 +21891,7 @@
         <v>27</v>
       </c>
       <c r="GI24" s="3" t="n">
-        <v>0.9558</v>
+        <v>0.9557</v>
       </c>
       <c r="GJ24" s="3" t="n">
         <v>0.1312</v>
@@ -21944,19 +21944,19 @@
         <v>6.62</v>
       </c>
       <c r="GZ24" s="3" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="HA24" s="3" t="n">
         <v>8.880000000000001</v>
       </c>
       <c r="HB24" s="3" t="n">
-        <v>16.54</v>
+        <v>16.52</v>
       </c>
       <c r="HC24" s="3" t="n">
         <v>3.8</v>
       </c>
       <c r="HD24" s="3" t="n">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="HE24" s="4" t="inlineStr">
         <is>
@@ -21964,16 +21964,16 @@
         </is>
       </c>
       <c r="HF24" s="3" t="n">
-        <v>62.4</v>
+        <v>62.5</v>
       </c>
       <c r="HG24" s="3" t="n">
-        <v>62.4</v>
+        <v>62.5</v>
       </c>
       <c r="HH24" s="3" t="n">
-        <v>54.5</v>
+        <v>54.6</v>
       </c>
       <c r="HI24" s="3" t="n">
-        <v>54.5</v>
+        <v>54.6</v>
       </c>
       <c r="HJ24" s="3" t="n">
         <v>49.1</v>
@@ -21982,10 +21982,10 @@
         <v>49.1</v>
       </c>
       <c r="HL24" s="3" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="HM24" s="3" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="HN24" s="3" t="n">
         <v>37.3</v>
@@ -21997,16 +21997,16 @@
         <v>30.7</v>
       </c>
       <c r="HQ24" s="3" t="n">
-        <v>27.1</v>
+        <v>27.2</v>
       </c>
       <c r="HR24" s="3" t="n">
-        <v>27.1</v>
+        <v>27.2</v>
       </c>
       <c r="HS24" s="3" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="HT24" s="3" t="n">
-        <v>23.7</v>
+        <v>23.8</v>
       </c>
       <c r="HU24" s="3" t="n">
         <v>20.9</v>
@@ -22021,10 +22021,10 @@
         <v>19.2</v>
       </c>
       <c r="HY24" s="3" t="n">
-        <v>17.4</v>
+        <v>17.5</v>
       </c>
       <c r="HZ24" s="3" t="n">
-        <v>17.4</v>
+        <v>17.5</v>
       </c>
       <c r="IA24" s="3" t="n">
         <v>16.2</v>
@@ -22033,16 +22033,16 @@
         <v>16.2</v>
       </c>
       <c r="IC24" s="3" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="ID24" s="3" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="IE24" s="3" t="n">
-        <v>12.6</v>
+        <v>12.8</v>
       </c>
       <c r="IF24" s="3" t="n">
-        <v>12.6</v>
+        <v>12.8</v>
       </c>
       <c r="IG24" s="3" t="n">
         <v>0</v>
@@ -23258,7 +23258,7 @@
         <v>158</v>
       </c>
       <c r="CL26" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CM26" s="4" t="inlineStr">
         <is>
@@ -25006,7 +25006,7 @@
         <v>158</v>
       </c>
       <c r="CL28" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CM28" s="4" t="inlineStr">
         <is>

</xml_diff>